<commit_message>
Add affiliate tag elevaonline-21 to all 250 product links
</commit_message>
<xml_diff>
--- a/generator/affiliate_links.xlsx
+++ b/generator/affiliate_links.xlsx
@@ -569,7 +569,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Air+Fryer+MAX+PRO+62L+AF180UK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
@@ -609,7 +613,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Foodi+Dual+Zone+76L+AF300UK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
@@ -649,7 +657,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tower+Vortx+4L+T17087&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
@@ -689,7 +701,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tefal+Easy+Fry+Dual+XXL+11L+EY942BG0&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -729,7 +745,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+3000+Series+Airfryer+L+NA23100&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
@@ -769,7 +789,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tower+Vortx+4L+T17087&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
@@ -809,7 +833,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=COSORI+47L+Pro+LE&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
@@ -849,7 +877,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Salter+EK4548+XL+8L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
@@ -889,7 +921,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Russell+Hobbs+SatisFry+Air+5L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
@@ -929,7 +965,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Air+Fryer+38L+AF100UK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
@@ -969,7 +1009,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Foodi+Dual+Zone+76L+AF300UK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1009,7 +1053,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Double+Stack+XL+95L+SL400UK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1049,7 +1097,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tefal+Easy+Fry+Dual+XXL+11L+EY942BG0&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1089,7 +1141,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tower+Vortx+Eco+Dual+Drawer+85L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1129,7 +1185,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Instant+Vortex+Plus+VersaZone+85L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1169,7 +1229,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Double+Stack+XL+95L+SL400UK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1209,7 +1273,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tefal+Easy+Fry+Dual+XXL+11L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1249,7 +1317,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Foodi+MAX+15in1+SmartLid+75L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1289,7 +1361,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Salter+Fuzion+Dual+9L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1329,7 +1405,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tower+Vortx+Vizion+14L+Air+Fryer+Oven&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1369,7 +1449,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninja+Air+Fryer+38L+AF100UK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1409,7 +1493,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=COSORI+Mini+21L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1449,7 +1537,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tower+Vortx+Compact+22L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1489,7 +1581,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+1000+Series+42L+NA12000&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1529,7 +1625,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Instant+Vortex+Slim+57L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1569,7 +1669,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+Series+800i+AC085011&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1609,7 +1713,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Levoit+Core+300S&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1649,7 +1757,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dyson+Purifier+Cool+TP07&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1689,7 +1801,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr"/>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Levoit+Core+600S&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1729,7 +1845,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Blueair+Blue+Max+3250i&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1769,7 +1889,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr"/>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+Series+800i+Allergy&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1809,7 +1933,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Levoit+Core+300S+Pet++Pollen&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1849,7 +1977,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Blueair+Blue+Max+3250i+Allergy&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1889,7 +2021,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dyson+Purifier+Cool+TP07+Allergy&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1929,7 +2065,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Vax+Pure+Air+300&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1969,7 +2109,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Blueair+Blue+Max+3250i+Sleep&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
@@ -2009,7 +2153,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+Series+800i+Sleep&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
@@ -2049,7 +2197,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Levoit+Core+300S+Sleep&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2089,7 +2241,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Smart+Air+Purifier+4+Compact+Sleep&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
@@ -2129,7 +2285,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Molekule+Air+Mini+Sleep&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2169,7 +2329,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Levoit+Core+600S+Large&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
@@ -2209,7 +2373,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+Series+3200+AC322010&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
@@ -2249,7 +2417,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Blueair+Blue+Max+3450i&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
@@ -2289,7 +2461,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Smart+Air+Purifier+4+Pro&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2329,7 +2505,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Shark+NeverChange+Air+Purifier+MAX&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
@@ -2369,7 +2549,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+Series+800i&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2409,7 +2593,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Levoit+Core+300S&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
@@ -2449,7 +2637,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Levoit+Core+MiniP&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
@@ -2489,7 +2681,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I50" s="4" t="inlineStr"/>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Smart+Air+Purifier+4+Compact&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2529,7 +2725,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+5in1+HEPA+Purifier&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2569,7 +2769,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I52" s="4" t="inlineStr"/>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Magnifica+S+ECAM22110B&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
@@ -2609,7 +2813,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I53" s="4" t="inlineStr"/>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Sage+Bambino+Plus&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2649,7 +2857,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I54" s="4" t="inlineStr"/>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Nespresso+Vertuo+Pop+by+Krups&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
@@ -2689,7 +2901,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I55" s="4" t="inlineStr"/>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Gaggia+Classic+Evo+Pro&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
@@ -2729,7 +2945,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr"/>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+2200+LatteGo&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
@@ -2769,7 +2989,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I57" s="4" t="inlineStr"/>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Magnifica+S+B2C&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
@@ -2809,7 +3033,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I58" s="4" t="inlineStr"/>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Philips+3200+LatteGo&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
@@ -2849,7 +3077,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Dinamica+Plus&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2889,7 +3121,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I60" s="4" t="inlineStr"/>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Jura+E6+Platin&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
@@ -2929,7 +3165,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I61" s="4" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Melitta+Caffeo+Solo&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
@@ -2969,7 +3209,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Nespresso+Vertuo+Pop+Budget&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
@@ -3009,7 +3253,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Stilosa+EC260&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
@@ -3049,7 +3297,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I64" s="4" t="inlineStr"/>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Melitta+Look+V+Timer+Filter&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
@@ -3089,7 +3341,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I65" s="4" t="inlineStr"/>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=AeroPress++JX+Manual+Grinder+bundle&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
@@ -3129,7 +3385,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I66" s="4" t="inlineStr"/>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tassimo+by+Bosch+Style&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J66" s="5" t="inlineStr"/>
     </row>
     <row r="67">
@@ -3169,7 +3429,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Nespresso+Essenza+Mini+Original&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J67" s="5" t="inlineStr"/>
     </row>
     <row r="68">
@@ -3209,7 +3473,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I68" s="4" t="inlineStr"/>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Nespresso+Vertuo+Next&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
@@ -3249,7 +3517,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I69" s="4" t="inlineStr"/>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=LOR+Barista+Sublime&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
@@ -3289,7 +3561,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I70" s="4" t="inlineStr"/>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Nescaf+Dolce+Gusto+Genio+S+Plus&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J70" s="5" t="inlineStr"/>
     </row>
     <row r="71">
@@ -3329,7 +3605,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I71" s="4" t="inlineStr"/>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Nespresso+Creatista+Plus+by+Sage&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
@@ -3369,7 +3649,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I72" s="4" t="inlineStr"/>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Sage+Bambino+Plus+Beginner&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
@@ -3409,7 +3693,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I73" s="4" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Dedica+Style+EC685&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
@@ -3449,7 +3737,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I74" s="4" t="inlineStr"/>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Gaggia+Classic+Evo+Pro+Beginner&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J74" s="5" t="inlineStr"/>
     </row>
     <row r="75">
@@ -3489,7 +3781,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I75" s="4" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Stilosa+Beginner&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J75" s="5" t="inlineStr"/>
     </row>
     <row r="76">
@@ -3529,7 +3825,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I76" s="4" t="inlineStr"/>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Sage+Barista+Express&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
@@ -3569,7 +3869,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I77" s="4" t="inlineStr"/>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=MeacoDry+Arete+One+12L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
@@ -3609,7 +3913,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I78" s="4" t="inlineStr"/>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Meaco+Low+Energy+20L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
@@ -3649,7 +3957,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I79" s="4" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+12L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
@@ -3689,7 +4001,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I80" s="4" t="inlineStr"/>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=EcoAir+DD1+Simple+MK3+Desiccant&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
@@ -3729,7 +4045,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I81" s="4" t="inlineStr"/>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=ElectriQ+CD12PROLE&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
@@ -3769,7 +4089,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I82" s="4" t="inlineStr"/>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=MeacoDry+Arete+One+10L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
@@ -3809,7 +4133,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I83" s="4" t="inlineStr"/>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+500ml+Mini&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
@@ -3849,7 +4177,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I84" s="4" t="inlineStr"/>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=EcoAir+DD1+Simple+MK3&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
@@ -3889,7 +4221,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I85" s="4" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Russell+Hobbs+RHDH1101&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
@@ -3929,7 +4265,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I86" s="4" t="inlineStr"/>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Duux+Bora+Smart+20L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
@@ -3969,7 +4309,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I87" s="4" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Meaco+Low+Energy+25L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J87" s="5" t="inlineStr"/>
     </row>
     <row r="88">
@@ -4009,7 +4353,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I88" s="4" t="inlineStr"/>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Meaco+Low+Energy+20L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
@@ -4049,7 +4397,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I89" s="4" t="inlineStr"/>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=ElectriQ+CD25PROLEV2&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
@@ -4089,7 +4441,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I90" s="4" t="inlineStr"/>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+20L+Premium&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
@@ -4129,7 +4485,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I91" s="4" t="inlineStr"/>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Inventor+Eva+Ion+Pro+20L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J91" s="5" t="inlineStr"/>
     </row>
     <row r="92">
@@ -4169,7 +4529,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I92" s="4" t="inlineStr"/>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Meaco+Low+Energy+20L+Laundry&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J92" s="5" t="inlineStr"/>
     </row>
     <row r="93">
@@ -4209,7 +4573,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I93" s="4" t="inlineStr"/>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=MeacoDry+Arete+One+12L+Laundry&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J93" s="5" t="inlineStr"/>
     </row>
     <row r="94">
@@ -4249,7 +4617,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I94" s="4" t="inlineStr"/>
+      <c r="I94" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=EcoAir+DD1+Simple+MK3+Laundry&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J94" s="5" t="inlineStr"/>
     </row>
     <row r="95">
@@ -4289,7 +4661,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I95" s="4" t="inlineStr"/>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+20L+Premium+Laundry&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J95" s="5" t="inlineStr"/>
     </row>
     <row r="96">
@@ -4329,7 +4705,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I96" s="4" t="inlineStr"/>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Vax+Power+Extract+18L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J96" s="5" t="inlineStr"/>
     </row>
     <row r="97">
@@ -4369,7 +4749,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I97" s="4" t="inlineStr"/>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=MeacoDry+Arete+One+20L&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J97" s="5" t="inlineStr"/>
     </row>
     <row r="98">
@@ -4409,7 +4793,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I98" s="4" t="inlineStr"/>
+      <c r="I98" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=ElectriQ+CD20PROLEV2+UV&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J98" s="5" t="inlineStr"/>
     </row>
     <row r="99">
@@ -4449,7 +4837,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Meaco+Low+Energy+25L+Damp+Rescue&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J99" s="5" t="inlineStr"/>
     </row>
     <row r="100">
@@ -4489,7 +4881,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I100" s="4" t="inlineStr"/>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+12L+Compressor+Starter&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J100" s="5" t="inlineStr"/>
     </row>
     <row r="101">
@@ -4529,7 +4925,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I101" s="4" t="inlineStr"/>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ionmax+ION632+Desiccant&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J101" s="5" t="inlineStr"/>
     </row>
     <row r="102">
@@ -4569,7 +4969,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I102" s="4" t="inlineStr"/>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Decathlon+Btwin+LD+920+E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J102" s="5" t="inlineStr"/>
     </row>
     <row r="103">
@@ -4609,7 +5013,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I103" s="4" t="inlineStr"/>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Engwe+P20&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J103" s="5" t="inlineStr"/>
     </row>
     <row r="104">
@@ -4649,7 +5057,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I104" s="4" t="inlineStr"/>
+      <c r="I104" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Cube+Touring+Hybrid+One+500&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J104" s="5" t="inlineStr"/>
     </row>
     <row r="105">
@@ -4689,7 +5101,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I105" s="4" t="inlineStr"/>
+      <c r="I105" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Fiido+D11&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J105" s="5" t="inlineStr"/>
     </row>
     <row r="106">
@@ -4729,7 +5145,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I106" s="4" t="inlineStr"/>
+      <c r="I106" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Trek+FX+2&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J106" s="5" t="inlineStr"/>
     </row>
     <row r="107">
@@ -4769,7 +5189,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I107" s="4" t="inlineStr"/>
+      <c r="I107" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Engwe+P20&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J107" s="5" t="inlineStr"/>
     </row>
     <row r="108">
@@ -4809,7 +5233,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I108" s="4" t="inlineStr"/>
+      <c r="I108" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Eleglide+M1+Plus&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J108" s="5" t="inlineStr"/>
     </row>
     <row r="109">
@@ -4849,7 +5277,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I109" s="4" t="inlineStr"/>
+      <c r="I109" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Fiido+D11&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J109" s="5" t="inlineStr"/>
     </row>
     <row r="110">
@@ -4889,7 +5321,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I110" s="4" t="inlineStr"/>
+      <c r="I110" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Decathlon+Btwin+EFold+500&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J110" s="5" t="inlineStr"/>
     </row>
     <row r="111">
@@ -4929,7 +5365,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I111" s="4" t="inlineStr"/>
+      <c r="I111" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=ADO+Air+20&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J111" s="5" t="inlineStr"/>
     </row>
     <row r="112">
@@ -4969,7 +5409,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I112" s="4" t="inlineStr"/>
+      <c r="I112" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=ADO+Air+20&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J112" s="5" t="inlineStr"/>
     </row>
     <row r="113">
@@ -5009,7 +5453,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I113" s="4" t="inlineStr"/>
+      <c r="I113" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Brompton+Electric+C+Line&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J113" s="5" t="inlineStr"/>
     </row>
     <row r="114">
@@ -5049,7 +5497,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I114" s="4" t="inlineStr"/>
+      <c r="I114" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Fiido+X&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J114" s="5" t="inlineStr"/>
     </row>
     <row r="115">
@@ -5089,7 +5541,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I115" s="4" t="inlineStr"/>
+      <c r="I115" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Decathlon+Btwin+EFold+900&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J115" s="5" t="inlineStr"/>
     </row>
     <row r="116">
@@ -5129,7 +5585,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I116" s="4" t="inlineStr"/>
+      <c r="I116" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Engwe+C20+Pro&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J116" s="5" t="inlineStr"/>
     </row>
     <row r="117">
@@ -5169,7 +5629,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I117" s="4" t="inlineStr"/>
+      <c r="I117" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Decathlon+Rockrider+EEXPL+520&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J117" s="5" t="inlineStr"/>
     </row>
     <row r="118">
@@ -5209,7 +5673,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I118" s="4" t="inlineStr"/>
+      <c r="I118" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Cube+Reaction+Hybrid+Performance+625&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J118" s="5" t="inlineStr"/>
     </row>
     <row r="119">
@@ -5249,7 +5717,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I119" s="4" t="inlineStr"/>
+      <c r="I119" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Giant+Talon+E+3&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J119" s="5" t="inlineStr"/>
     </row>
     <row r="120">
@@ -5289,7 +5761,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I120" s="4" t="inlineStr"/>
+      <c r="I120" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Engwe+Engine+Pro+20&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J120" s="5" t="inlineStr"/>
     </row>
     <row r="121">
@@ -5329,7 +5805,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I121" s="4" t="inlineStr"/>
+      <c r="I121" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Specialized+Turbo+Tero+30&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J121" s="5" t="inlineStr"/>
     </row>
     <row r="122">
@@ -5369,7 +5849,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I122" s="4" t="inlineStr"/>
+      <c r="I122" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Decathlon+Btwin+LD+920+E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J122" s="5" t="inlineStr"/>
     </row>
     <row r="123">
@@ -5409,7 +5893,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I123" s="4" t="inlineStr"/>
+      <c r="I123" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Cube+Touring+Hybrid+One+500&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J123" s="5" t="inlineStr"/>
     </row>
     <row r="124">
@@ -5449,7 +5937,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I124" s="4" t="inlineStr"/>
+      <c r="I124" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Gazelle+Paris+C7+HMB&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J124" s="5" t="inlineStr"/>
     </row>
     <row r="125">
@@ -5489,7 +5981,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I125" s="4" t="inlineStr"/>
+      <c r="I125" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Eleglide+T1+StepThru&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J125" s="5" t="inlineStr"/>
     </row>
     <row r="126">
@@ -5529,7 +6025,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I126" s="4" t="inlineStr"/>
+      <c r="I126" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Tenways+CGO600+Pro&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J126" s="5" t="inlineStr"/>
     </row>
     <row r="127">
@@ -5569,7 +6069,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I127" s="4" t="inlineStr"/>
+      <c r="I127" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Dragon+4+25kW+Oil+Radiator+TRD41025T&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J127" s="5" t="inlineStr"/>
     </row>
     <row r="128">
@@ -5609,7 +6113,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I128" s="4" t="inlineStr"/>
+      <c r="I128" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dyson+HotCool+Jet+Focus+AM09&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J128" s="5" t="inlineStr"/>
     </row>
     <row r="129">
@@ -5649,7 +6157,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I129" s="4" t="inlineStr"/>
+      <c r="I129" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+2kW+Ceramic+Fan+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J129" s="5" t="inlineStr"/>
     </row>
     <row r="130">
@@ -5689,7 +6201,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I130" s="4" t="inlineStr"/>
+      <c r="I130" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Stiebel+Eltron+CK+20+S+Wall+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J130" s="5" t="inlineStr"/>
     </row>
     <row r="131">
@@ -5729,7 +6245,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I131" s="4" t="inlineStr"/>
+      <c r="I131" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Devola+2kW+Smart+Glass+Panel+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J131" s="5" t="inlineStr"/>
     </row>
     <row r="132">
@@ -5769,7 +6289,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I132" s="4" t="inlineStr"/>
+      <c r="I132" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Vonhaus+550W+Glass+Panel+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J132" s="5" t="inlineStr"/>
     </row>
     <row r="133">
@@ -5809,7 +6333,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I133" s="4" t="inlineStr"/>
+      <c r="I133" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+1200W+Halogen+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J133" s="5" t="inlineStr"/>
     </row>
     <row r="134">
@@ -5849,7 +6377,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I134" s="4" t="inlineStr"/>
+      <c r="I134" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Duronic+HV052+UnderDesk+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J134" s="5" t="inlineStr"/>
     </row>
     <row r="135">
@@ -5889,7 +6421,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I135" s="4" t="inlineStr"/>
+      <c r="I135" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Radia+S+15kW+Oil+Radiator+TRRS0715&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J135" s="5" t="inlineStr"/>
     </row>
     <row r="136">
@@ -5929,7 +6465,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I136" s="4" t="inlineStr"/>
+      <c r="I136" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Devola+15kW+Smart+WiFi+Panel&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J136" s="5" t="inlineStr"/>
     </row>
     <row r="137">
@@ -5969,7 +6509,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I137" s="4" t="inlineStr"/>
+      <c r="I137" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Dragon+4+25kW+TRD41025T&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J137" s="5" t="inlineStr"/>
     </row>
     <row r="138">
@@ -6009,7 +6553,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I138" s="4" t="inlineStr"/>
+      <c r="I138" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+25kW+Digital+Oil+Radiator&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J138" s="5" t="inlineStr"/>
     </row>
     <row r="139">
@@ -6049,7 +6597,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I139" s="4" t="inlineStr"/>
+      <c r="I139" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dimplex+2kW+ECR20Tie+Cadiz&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J139" s="5" t="inlineStr"/>
     </row>
     <row r="140">
@@ -6089,7 +6641,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I140" s="4" t="inlineStr"/>
+      <c r="I140" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=VonHaus+15kW+7Fin+Oil+Radiator&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J140" s="5" t="inlineStr"/>
     </row>
     <row r="141">
@@ -6129,7 +6685,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I141" s="4" t="inlineStr"/>
+      <c r="I141" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=DeLonghi+Radia+S+2kW+with+Timer+TRRS0920T&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J141" s="5" t="inlineStr"/>
     </row>
     <row r="142">
@@ -6169,7 +6729,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I142" s="4" t="inlineStr"/>
+      <c r="I142" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Devola+2kW+Smart+Glass+Panel&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J142" s="5" t="inlineStr"/>
     </row>
     <row r="143">
@@ -6209,7 +6773,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I143" s="4" t="inlineStr"/>
+      <c r="I143" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Mylek+15kW+Smart+Panel&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J143" s="5" t="inlineStr"/>
     </row>
     <row r="144">
@@ -6249,7 +6817,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I144" s="4" t="inlineStr"/>
+      <c r="I144" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dimplex+DTD4W20+Panel+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J144" s="5" t="inlineStr"/>
     </row>
     <row r="145">
@@ -6289,7 +6861,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I145" s="4" t="inlineStr"/>
+      <c r="I145" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Princess+15kW+Smart+Glass+Panel&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J145" s="5" t="inlineStr"/>
     </row>
     <row r="146">
@@ -6329,7 +6905,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I146" s="4" t="inlineStr"/>
+      <c r="I146" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Warmlite+1kW+Slim+Panel&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J146" s="5" t="inlineStr"/>
     </row>
     <row r="147">
@@ -6369,7 +6949,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I147" s="4" t="inlineStr"/>
+      <c r="I147" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Stiebel+Eltron+CK+20+S&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J147" s="5" t="inlineStr"/>
     </row>
     <row r="148">
@@ -6409,7 +6993,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I148" s="4" t="inlineStr"/>
+      <c r="I148" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pro+Breeze+2kW+Mini+Ceramic&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J148" s="5" t="inlineStr"/>
     </row>
     <row r="149">
@@ -6449,7 +7037,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I149" s="4" t="inlineStr"/>
+      <c r="I149" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dimplex+2kW+Downflow+Bathroom+Heater+FX20VE&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J149" s="5" t="inlineStr"/>
     </row>
     <row r="150">
@@ -6489,7 +7081,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I150" s="4" t="inlineStr"/>
+      <c r="I150" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Devola+550W+Towel+Rail++Timer&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J150" s="5" t="inlineStr"/>
     </row>
     <row r="151">
@@ -6529,7 +7125,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I151" s="4" t="inlineStr"/>
+      <c r="I151" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=VonHaus+18kW+Wall+Ceramic+Heater&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J151" s="5" t="inlineStr"/>
     </row>
     <row r="152">
@@ -6569,7 +7169,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I152" s="4" t="inlineStr"/>
+      <c r="I152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Electric+Scooter+4+Pro+2nd+Gen&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J152" s="5" t="inlineStr"/>
     </row>
     <row r="153">
@@ -6609,7 +7213,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I153" s="4" t="inlineStr"/>
+      <c r="I153" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Ninebot+MAX+G2+E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J153" s="5" t="inlineStr"/>
     </row>
     <row r="154">
@@ -6649,7 +7257,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I154" s="4" t="inlineStr"/>
+      <c r="I154" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Aovo+Pro+AP07&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J154" s="5" t="inlineStr"/>
     </row>
     <row r="155">
@@ -6689,7 +7301,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I155" s="4" t="inlineStr"/>
+      <c r="I155" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pure+Advance+Flex&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J155" s="5" t="inlineStr"/>
     </row>
     <row r="156">
@@ -6729,7 +7345,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I156" s="4" t="inlineStr"/>
+      <c r="I156" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ninebot+KickScooter+F2+E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J156" s="5" t="inlineStr"/>
     </row>
     <row r="157">
@@ -6769,7 +7389,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I157" s="4" t="inlineStr"/>
+      <c r="I157" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Electric+Scooter+4+Lite+2nd+Gen&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J157" s="5" t="inlineStr"/>
     </row>
     <row r="158">
@@ -6809,7 +7433,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I158" s="4" t="inlineStr"/>
+      <c r="I158" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Aovo+Pro+M365+Upgraded&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J158" s="5" t="inlineStr"/>
     </row>
     <row r="159">
@@ -6849,7 +7477,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I159" s="4" t="inlineStr"/>
+      <c r="I159" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Ninebot+E2+Pro+E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J159" s="5" t="inlineStr"/>
     </row>
     <row r="160">
@@ -6889,7 +7521,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I160" s="4" t="inlineStr"/>
+      <c r="I160" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=iScooter+i9+Max&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J160" s="5" t="inlineStr"/>
     </row>
     <row r="161">
@@ -6929,7 +7565,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I161" s="4" t="inlineStr"/>
+      <c r="I161" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Electric+Scooter+4+Standard&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J161" s="5" t="inlineStr"/>
     </row>
     <row r="162">
@@ -6969,7 +7609,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I162" s="4" t="inlineStr"/>
+      <c r="I162" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Ninebot+MAX+G3+E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J162" s="5" t="inlineStr"/>
     </row>
     <row r="163">
@@ -7009,7 +7653,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I163" s="4" t="inlineStr"/>
+      <c r="I163" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pure+Advance+&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J163" s="5" t="inlineStr"/>
     </row>
     <row r="164">
@@ -7049,7 +7697,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I164" s="4" t="inlineStr"/>
+      <c r="I164" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Electric+Scooter+5+Max&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J164" s="5" t="inlineStr"/>
     </row>
     <row r="165">
@@ -7089,7 +7741,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I165" s="4" t="inlineStr"/>
+      <c r="I165" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=NIU+KQi3+Max&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J165" s="5" t="inlineStr"/>
     </row>
     <row r="166">
@@ -7129,7 +7785,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I166" s="4" t="inlineStr"/>
+      <c r="I166" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=VMAX+VX2+Pro+GT&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J166" s="5" t="inlineStr"/>
     </row>
     <row r="167">
@@ -7169,7 +7829,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I167" s="4" t="inlineStr"/>
+      <c r="I167" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Mi+Electric+Scooter+3+Lite&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J167" s="5" t="inlineStr"/>
     </row>
     <row r="168">
@@ -7209,7 +7873,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I168" s="4" t="inlineStr"/>
+      <c r="I168" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Ninebot+Air+T15E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J168" s="5" t="inlineStr"/>
     </row>
     <row r="169">
@@ -7249,7 +7917,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I169" s="4" t="inlineStr"/>
+      <c r="I169" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Pure+Air4&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J169" s="5" t="inlineStr"/>
     </row>
     <row r="170">
@@ -7289,7 +7961,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I170" s="4" t="inlineStr"/>
+      <c r="I170" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=iScooter+i8&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J170" s="5" t="inlineStr"/>
     </row>
     <row r="171">
@@ -7329,7 +8005,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I171" s="4" t="inlineStr"/>
+      <c r="I171" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=ducati+ProI+Evo+Safe+Ride&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J171" s="5" t="inlineStr"/>
     </row>
     <row r="172">
@@ -7369,7 +8049,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I172" s="4" t="inlineStr"/>
+      <c r="I172" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Ninebot+MAX+G2+E+120+kg&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J172" s="5" t="inlineStr"/>
     </row>
     <row r="173">
@@ -7409,7 +8093,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I173" s="4" t="inlineStr"/>
+      <c r="I173" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=VMAX+VX2+Pro+ST&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J173" s="5" t="inlineStr"/>
     </row>
     <row r="174">
@@ -7449,7 +8137,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I174" s="4" t="inlineStr"/>
+      <c r="I174" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Electric+Scooter+5+Max+118+kg&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J174" s="5" t="inlineStr"/>
     </row>
     <row r="175">
@@ -7489,7 +8181,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I175" s="4" t="inlineStr"/>
+      <c r="I175" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=NIU+KQi+300X&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J175" s="5" t="inlineStr"/>
     </row>
     <row r="176">
@@ -7529,7 +8225,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I176" s="4" t="inlineStr"/>
+      <c r="I176" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=iScooter+iX4&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J176" s="5" t="inlineStr"/>
     </row>
     <row r="177">
@@ -7569,7 +8269,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I177" s="4" t="inlineStr"/>
+      <c r="I177" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=SIHOO+Doro+C300&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J177" s="5" t="inlineStr"/>
     </row>
     <row r="178">
@@ -7609,7 +8313,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I178" s="4" t="inlineStr"/>
+      <c r="I178" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Herman+Miller+Aeron+Remastered&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J178" s="5" t="inlineStr"/>
     </row>
     <row r="179">
@@ -7649,7 +8357,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I179" s="4" t="inlineStr"/>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Steelcase+Series+1&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J179" s="5" t="inlineStr"/>
     </row>
     <row r="180">
@@ -7689,7 +8401,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I180" s="4" t="inlineStr"/>
+      <c r="I180" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flexispot+BS11+Pro+C7&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J180" s="5" t="inlineStr"/>
     </row>
     <row r="181">
@@ -7729,7 +8445,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I181" s="4" t="inlineStr"/>
+      <c r="I181" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=IKEA+MARKUS&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J181" s="5" t="inlineStr"/>
     </row>
     <row r="182">
@@ -7769,7 +8489,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I182" s="4" t="inlineStr"/>
+      <c r="I182" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=IKEA+MARKUS+Budget&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J182" s="5" t="inlineStr"/>
     </row>
     <row r="183">
@@ -7809,7 +8533,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I183" s="4" t="inlineStr"/>
+      <c r="I183" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=SIHOO+M18&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J183" s="5" t="inlineStr"/>
     </row>
     <row r="184">
@@ -7849,7 +8577,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I184" s="4" t="inlineStr"/>
+      <c r="I184" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Songmics+OBN37BK&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J184" s="5" t="inlineStr"/>
     </row>
     <row r="185">
@@ -7889,7 +8621,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I185" s="4" t="inlineStr"/>
+      <c r="I185" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flexispot+OC3&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J185" s="5" t="inlineStr"/>
     </row>
     <row r="186">
@@ -7929,7 +8665,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I186" s="4" t="inlineStr"/>
+      <c r="I186" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=HBADA+E1+Ergonomic&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J186" s="5" t="inlineStr"/>
     </row>
     <row r="187">
@@ -7969,7 +8709,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I187" s="4" t="inlineStr"/>
+      <c r="I187" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flexispot+E7+Pro&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J187" s="5" t="inlineStr"/>
     </row>
     <row r="188">
@@ -8009,7 +8753,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I188" s="4" t="inlineStr"/>
+      <c r="I188" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=IKEA+TROTTEN+Electric+manual+crank&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J188" s="5" t="inlineStr"/>
     </row>
     <row r="189">
@@ -8049,7 +8797,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I189" s="4" t="inlineStr"/>
+      <c r="I189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flexispot+E7&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J189" s="5" t="inlineStr"/>
     </row>
     <row r="190">
@@ -8089,7 +8841,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I190" s="4" t="inlineStr"/>
+      <c r="I190" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Songmics+LSD012+Electric&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J190" s="5" t="inlineStr"/>
     </row>
     <row r="191">
@@ -8129,7 +8885,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I191" s="4" t="inlineStr"/>
+      <c r="I191" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Secretlab+MAGNUS+Pro++tabletop&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J191" s="5" t="inlineStr"/>
     </row>
     <row r="192">
@@ -8169,7 +8929,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I192" s="4" t="inlineStr"/>
+      <c r="I192" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flexispot+E7++10060+top&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J192" s="5" t="inlineStr"/>
     </row>
     <row r="193">
@@ -8209,7 +8973,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I193" s="4" t="inlineStr"/>
+      <c r="I193" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=IKEA+MICKE+10550&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J193" s="5" t="inlineStr"/>
     </row>
     <row r="194">
@@ -8249,7 +9017,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I194" s="4" t="inlineStr"/>
+      <c r="I194" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Habitat+Compton+Folding+Desk&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J194" s="5" t="inlineStr"/>
     </row>
     <row r="195">
@@ -8289,7 +9061,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I195" s="4" t="inlineStr"/>
+      <c r="I195" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=VASAGLE+LShaped+Corner+Desk+130&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J195" s="5" t="inlineStr"/>
     </row>
     <row r="196">
@@ -8329,7 +9105,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I196" s="4" t="inlineStr"/>
+      <c r="I196" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=String+Furniture+Works+Wall+Desk+78&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J196" s="5" t="inlineStr"/>
     </row>
     <row r="197">
@@ -8369,7 +9149,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I197" s="4" t="inlineStr"/>
+      <c r="I197" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flexispot+M7B+Converter+35&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J197" s="5" t="inlineStr"/>
     </row>
     <row r="198">
@@ -8409,7 +9193,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I198" s="4" t="inlineStr"/>
+      <c r="I198" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ergotron+LX+Monitor+Arm&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J198" s="5" t="inlineStr"/>
     </row>
     <row r="199">
@@ -8449,7 +9237,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I199" s="4" t="inlineStr"/>
+      <c r="I199" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=HUANUO+Dual+Monitor+Arm&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J199" s="5" t="inlineStr"/>
     </row>
     <row r="200">
@@ -8489,7 +9281,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I200" s="4" t="inlineStr"/>
+      <c r="I200" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Kensington+SoleMate+Pro+Footrest&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J200" s="5" t="inlineStr"/>
     </row>
     <row r="201">
@@ -8529,7 +9325,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I201" s="4" t="inlineStr"/>
+      <c r="I201" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Topo+AntiFatigue+Mat+by+Ergodriven&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J201" s="5" t="inlineStr"/>
     </row>
     <row r="202">
@@ -8569,7 +9369,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I202" s="4" t="inlineStr"/>
+      <c r="I202" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Navimow+i105E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J202" s="5" t="inlineStr"/>
     </row>
     <row r="203">
@@ -8609,7 +9413,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I203" s="4" t="inlineStr"/>
+      <c r="I203" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Husqvarna+Automower+305&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J203" s="5" t="inlineStr"/>
     </row>
     <row r="204">
@@ -8649,7 +9457,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I204" s="4" t="inlineStr"/>
+      <c r="I204" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Worx+Landroid+Vision+M600&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J204" s="5" t="inlineStr"/>
     </row>
     <row r="205">
@@ -8689,7 +9501,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I205" s="4" t="inlineStr"/>
+      <c r="I205" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Gardena+Sileno+City+250&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J205" s="5" t="inlineStr"/>
     </row>
     <row r="206">
@@ -8729,7 +9545,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I206" s="4" t="inlineStr"/>
+      <c r="I206" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Navimow+i110E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J206" s="5" t="inlineStr"/>
     </row>
     <row r="207">
@@ -8769,7 +9589,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I207" s="4" t="inlineStr"/>
+      <c r="I207" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Gardena+Sileno+City+250+Small&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J207" s="5" t="inlineStr"/>
     </row>
     <row r="208">
@@ -8809,7 +9633,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I208" s="4" t="inlineStr"/>
+      <c r="I208" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Navimow+i105E+Small&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J208" s="5" t="inlineStr"/>
     </row>
     <row r="209">
@@ -8849,7 +9677,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I209" s="4" t="inlineStr"/>
+      <c r="I209" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Worx+Landroid+S300&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J209" s="5" t="inlineStr"/>
     </row>
     <row r="210">
@@ -8889,7 +9721,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I210" s="4" t="inlineStr"/>
+      <c r="I210" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flymo+EasiLife+GO+250&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J210" s="5" t="inlineStr"/>
     </row>
     <row r="211">
@@ -8929,7 +9765,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I211" s="4" t="inlineStr"/>
+      <c r="I211" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Bosch+Indego+S+350&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J211" s="5" t="inlineStr"/>
     </row>
     <row r="212">
@@ -8969,7 +9809,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I212" s="4" t="inlineStr"/>
+      <c r="I212" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Navimow+i110E+Large&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J212" s="5" t="inlineStr"/>
     </row>
     <row r="213">
@@ -9009,7 +9853,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I213" s="4" t="inlineStr"/>
+      <c r="I213" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Husqvarna+Automower+430X+NERA&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J213" s="5" t="inlineStr"/>
     </row>
     <row r="214">
@@ -9049,7 +9897,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I214" s="4" t="inlineStr"/>
+      <c r="I214" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Navimow+H1500E&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J214" s="5" t="inlineStr"/>
     </row>
     <row r="215">
@@ -9089,7 +9941,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I215" s="4" t="inlineStr"/>
+      <c r="I215" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Worx+Landroid+L2000&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J215" s="5" t="inlineStr"/>
     </row>
     <row r="216">
@@ -9129,7 +9985,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I216" s="4" t="inlineStr"/>
+      <c r="I216" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ecovacs+Goat+G12000&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J216" s="5" t="inlineStr"/>
     </row>
     <row r="217">
@@ -9169,7 +10029,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I217" s="4" t="inlineStr"/>
+      <c r="I217" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Segway+Navimow+i105E+WireFree&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J217" s="5" t="inlineStr"/>
     </row>
     <row r="218">
@@ -9209,7 +10073,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I218" s="4" t="inlineStr"/>
+      <c r="I218" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Worx+Landroid+Vision+M600+WireFree&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J218" s="5" t="inlineStr"/>
     </row>
     <row r="219">
@@ -9249,7 +10117,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I219" s="4" t="inlineStr"/>
+      <c r="I219" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Husqvarna+Automower+320+NERA++EPOS&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J219" s="5" t="inlineStr"/>
     </row>
     <row r="220">
@@ -9289,7 +10161,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I220" s="4" t="inlineStr"/>
+      <c r="I220" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Ecovacs+Goat+G1800&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J220" s="5" t="inlineStr"/>
     </row>
     <row r="221">
@@ -9329,7 +10205,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I221" s="4" t="inlineStr"/>
+      <c r="I221" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Mammotion+Luba+2+AWD+1000&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J221" s="5" t="inlineStr"/>
     </row>
     <row r="222">
@@ -9369,7 +10249,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I222" s="4" t="inlineStr"/>
+      <c r="I222" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Gardena+Sileno+City+250+Budget&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J222" s="5" t="inlineStr"/>
     </row>
     <row r="223">
@@ -9409,7 +10293,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I223" s="4" t="inlineStr"/>
+      <c r="I223" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Flymo+EasiLife+GO+500&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J223" s="5" t="inlineStr"/>
     </row>
     <row r="224">
@@ -9449,7 +10337,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I224" s="4" t="inlineStr"/>
+      <c r="I224" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Worx+Landroid+S300+Budget&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J224" s="5" t="inlineStr"/>
     </row>
     <row r="225">
@@ -9489,7 +10381,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I225" s="4" t="inlineStr"/>
+      <c r="I225" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Yard+Force+Compact+300RBS&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J225" s="5" t="inlineStr"/>
     </row>
     <row r="226">
@@ -9529,7 +10425,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I226" s="4" t="inlineStr"/>
+      <c r="I226" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Einhell+FREELEXO+400m+BT&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J226" s="5" t="inlineStr"/>
     </row>
     <row r="227">
@@ -9569,7 +10469,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I227" s="4" t="inlineStr"/>
+      <c r="I227" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+Q8+Max&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J227" s="5" t="inlineStr"/>
     </row>
     <row r="228">
@@ -9609,7 +10513,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I228" s="4" t="inlineStr"/>
+      <c r="I228" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+S8+MaxV+Ultra&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J228" s="5" t="inlineStr"/>
     </row>
     <row r="229">
@@ -9649,7 +10557,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I229" s="4" t="inlineStr"/>
+      <c r="I229" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Eufy+RoboVac+11S+MAX&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J229" s="5" t="inlineStr"/>
     </row>
     <row r="230">
@@ -9689,7 +10601,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I230" s="4" t="inlineStr"/>
+      <c r="I230" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dreame+L10s+Ultra+Gen+2&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J230" s="5" t="inlineStr"/>
     </row>
     <row r="231">
@@ -9729,7 +10645,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I231" s="4" t="inlineStr"/>
+      <c r="I231" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=iRobot+Roomba+Combo+j7&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J231" s="5" t="inlineStr"/>
     </row>
     <row r="232">
@@ -9769,7 +10689,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I232" s="4" t="inlineStr"/>
+      <c r="I232" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+Q7+L5&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J232" s="5" t="inlineStr"/>
     </row>
     <row r="233">
@@ -9809,7 +10733,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I233" s="4" t="inlineStr"/>
+      <c r="I233" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Eufy+RoboVac+11S+MAX+Budget&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J233" s="5" t="inlineStr"/>
     </row>
     <row r="234">
@@ -9849,7 +10777,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I234" s="4" t="inlineStr"/>
+      <c r="I234" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dreame+D10+Plus+Gen+2&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J234" s="5" t="inlineStr"/>
     </row>
     <row r="235">
@@ -9889,7 +10821,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I235" s="4" t="inlineStr"/>
+      <c r="I235" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+Robot+Vacuum+S20&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J235" s="5" t="inlineStr"/>
     </row>
     <row r="236">
@@ -9929,7 +10865,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I236" s="4" t="inlineStr"/>
+      <c r="I236" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Lefant+M310&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J236" s="5" t="inlineStr"/>
     </row>
     <row r="237">
@@ -9969,7 +10909,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I237" s="4" t="inlineStr"/>
+      <c r="I237" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=iRobot+Roomba+Combo+j7+Pets&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J237" s="5" t="inlineStr"/>
     </row>
     <row r="238">
@@ -10009,7 +10953,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I238" s="4" t="inlineStr"/>
+      <c r="I238" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+Q8+Max+Pets&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J238" s="5" t="inlineStr"/>
     </row>
     <row r="239">
@@ -10049,7 +10997,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I239" s="4" t="inlineStr"/>
+      <c r="I239" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dreame+L10s+Ultra+Gen+2+Pets&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J239" s="5" t="inlineStr"/>
     </row>
     <row r="240">
@@ -10089,7 +11041,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I240" s="4" t="inlineStr"/>
+      <c r="I240" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Eufy+X10+Pro+Omni+Pets&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J240" s="5" t="inlineStr"/>
     </row>
     <row r="241">
@@ -10129,7 +11085,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I241" s="4" t="inlineStr"/>
+      <c r="I241" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Shark+Matrix+Plus+2in1+Pets&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J241" s="5" t="inlineStr"/>
     </row>
     <row r="242">
@@ -10169,7 +11129,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I242" s="4" t="inlineStr"/>
+      <c r="I242" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+S8+MaxV+Ultra+Mop&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J242" s="5" t="inlineStr"/>
     </row>
     <row r="243">
@@ -10209,7 +11173,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I243" s="4" t="inlineStr"/>
+      <c r="I243" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dreame+L10s+Ultra+Gen+2+Mop&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J243" s="5" t="inlineStr"/>
     </row>
     <row r="244">
@@ -10249,7 +11217,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I244" s="4" t="inlineStr"/>
+      <c r="I244" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Eufy+X10+Pro+Omni+Mop&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J244" s="5" t="inlineStr"/>
     </row>
     <row r="245">
@@ -10289,7 +11261,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I245" s="4" t="inlineStr"/>
+      <c r="I245" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+Q+Revo&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J245" s="5" t="inlineStr"/>
     </row>
     <row r="246">
@@ -10329,7 +11305,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I246" s="4" t="inlineStr"/>
+      <c r="I246" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Xiaomi+X20&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J246" s="5" t="inlineStr"/>
     </row>
     <row r="247">
@@ -10369,7 +11349,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I247" s="4" t="inlineStr"/>
+      <c r="I247" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+S8+MaxV+Ultra+Premium&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J247" s="5" t="inlineStr"/>
     </row>
     <row r="248">
@@ -10409,7 +11393,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I248" s="4" t="inlineStr"/>
+      <c r="I248" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Dreame+X40+Ultra&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J248" s="5" t="inlineStr"/>
     </row>
     <row r="249">
@@ -10449,7 +11437,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I249" s="4" t="inlineStr"/>
+      <c r="I249" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=iRobot+Roomba+j9+Combo&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J249" s="5" t="inlineStr"/>
     </row>
     <row r="250">
@@ -10489,7 +11481,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I250" s="4" t="inlineStr"/>
+      <c r="I250" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Eufy+Omni+S1+Pro&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J250" s="5" t="inlineStr"/>
     </row>
     <row r="251">
@@ -10529,7 +11525,11 @@
           <t>abrir produto →</t>
         </is>
       </c>
-      <c r="I251" s="4" t="inlineStr"/>
+      <c r="I251" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/s?k=Roborock+Q+Revo+Premium+Entry&amp;tag=elevaonline-21</t>
+        </is>
+      </c>
       <c r="J251" s="5" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>